<commit_message>
docs: integrazione release 1.53.1 - tabella dec use case
</commit_message>
<xml_diff>
--- a/docs/Decodifiche/3_dec_use_case.xlsx
+++ b/docs/Decodifiche/3_dec_use_case.xlsx
@@ -1973,7 +1973,7 @@
     <t>51112</t>
   </si>
   <si>
-    <t>Dichiarazione di volonta' d'acquisto della cittadinanza italiana di minore art.1-ter legge n.74/2025 (transitoria valida solo fino al 31 maggio 2026)</t>
+    <t>Dichiarazione di volonta' d'acquisto della cittadinanza italiana di minore art.1-ter legge n.74/2025 (transitoria valida solo fino al 31 maggio 2029)</t>
   </si>
   <si>
     <t>51201</t>
@@ -2123,7 +2123,7 @@
     <t>52156</t>
   </si>
   <si>
-    <t>Esito di accertamento per articolo 4 comma 1-bis</t>
+    <t>Esito di accertamento per articolo 4 comma 1-bis e art. 1.1 ter da consolato</t>
   </si>
   <si>
     <t>52157</t>

</xml_diff>

<commit_message>
docs: integrazione documentazione 1.53.1, dismissione casi uso 321321, 321421
</commit_message>
<xml_diff>
--- a/docs/Decodifiche/3_dec_use_case.xlsx
+++ b/docs/Decodifiche/3_dec_use_case.xlsx
@@ -1574,6 +1574,9 @@
     <t>Matrimonio con Rito Religioso Cattolico con Riconoscimento di uno o piu' figli</t>
   </si>
   <si>
+    <t>2025-01-01 00:00:00.0</t>
+  </si>
+  <si>
     <t>321411</t>
   </si>
   <si>
@@ -1872,9 +1875,6 @@
   </si>
   <si>
     <t>Trascrizione di sentenza straniera di scioglimento unione civile</t>
-  </si>
-  <si>
-    <t>2025-01-01 00:00:00.0</t>
   </si>
   <si>
     <t>449999</t>
@@ -7348,7 +7348,7 @@
         <v>8</v>
       </c>
       <c r="D251" s="2" t="s">
-        <v>9</v>
+        <v>520</v>
       </c>
       <c r="E251" s="2" t="s">
         <v>10</v>
@@ -7359,10 +7359,10 @@
     </row>
     <row r="252">
       <c r="A252" s="2" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="C252" s="2" t="s">
         <v>8</v>
@@ -7379,16 +7379,16 @@
     </row>
     <row r="253">
       <c r="A253" s="2" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="C253" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D253" s="2" t="s">
-        <v>9</v>
+        <v>520</v>
       </c>
       <c r="E253" s="2" t="s">
         <v>10</v>
@@ -7399,10 +7399,10 @@
     </row>
     <row r="254">
       <c r="A254" s="2" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B254" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="C254" s="2" t="s">
         <v>321</v>
@@ -7419,10 +7419,10 @@
     </row>
     <row r="255">
       <c r="A255" s="2" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="C255" s="2" t="s">
         <v>321</v>
@@ -7439,10 +7439,10 @@
     </row>
     <row r="256">
       <c r="A256" s="2" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="C256" s="2" t="s">
         <v>8</v>
@@ -7459,10 +7459,10 @@
     </row>
     <row r="257">
       <c r="A257" s="2" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="C257" s="2" t="s">
         <v>8</v>
@@ -7479,10 +7479,10 @@
     </row>
     <row r="258">
       <c r="A258" s="2" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="C258" s="2" t="s">
         <v>8</v>
@@ -7499,10 +7499,10 @@
     </row>
     <row r="259">
       <c r="A259" s="2" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="C259" s="2" t="s">
         <v>8</v>
@@ -7519,10 +7519,10 @@
     </row>
     <row r="260">
       <c r="A260" s="2" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="C260" s="2" t="s">
         <v>8</v>
@@ -7539,10 +7539,10 @@
     </row>
     <row r="261">
       <c r="A261" s="2" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C261" s="2" t="s">
         <v>8</v>
@@ -7559,13 +7559,13 @@
     </row>
     <row r="262">
       <c r="A262" s="2" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="D262" s="2" t="s">
         <v>9</v>
@@ -7579,10 +7579,10 @@
     </row>
     <row r="263">
       <c r="A263" s="2" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C263" s="2" t="s">
         <v>8</v>
@@ -7599,10 +7599,10 @@
     </row>
     <row r="264">
       <c r="A264" s="2" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="C264" s="2" t="s">
         <v>8</v>
@@ -7619,10 +7619,10 @@
     </row>
     <row r="265">
       <c r="A265" s="2" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="C265" s="2" t="s">
         <v>8</v>
@@ -7639,10 +7639,10 @@
     </row>
     <row r="266">
       <c r="A266" s="2" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C266" s="2" t="s">
         <v>8</v>
@@ -7659,10 +7659,10 @@
     </row>
     <row r="267">
       <c r="A267" s="2" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C267" s="2" t="s">
         <v>8</v>
@@ -7679,10 +7679,10 @@
     </row>
     <row r="268">
       <c r="A268" s="2" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="C268" s="2" t="s">
         <v>8</v>
@@ -7699,10 +7699,10 @@
     </row>
     <row r="269">
       <c r="A269" s="2" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="C269" s="2" t="s">
         <v>8</v>
@@ -7719,10 +7719,10 @@
     </row>
     <row r="270">
       <c r="A270" s="2" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C270" s="2" t="s">
         <v>8</v>
@@ -7739,16 +7739,16 @@
     </row>
     <row r="271">
       <c r="A271" s="2" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C271" s="2" t="s">
         <v>321</v>
       </c>
       <c r="D271" s="2" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="E271" s="2" t="s">
         <v>10</v>
@@ -7759,10 +7759,10 @@
     </row>
     <row r="272">
       <c r="A272" s="2" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="C272" s="2" t="s">
         <v>8</v>
@@ -7779,10 +7779,10 @@
     </row>
     <row r="273">
       <c r="A273" s="2" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C273" s="2" t="s">
         <v>8</v>
@@ -7799,10 +7799,10 @@
     </row>
     <row r="274">
       <c r="A274" s="2" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C274" s="2" t="s">
         <v>8</v>
@@ -7819,13 +7819,13 @@
     </row>
     <row r="275">
       <c r="A275" s="2" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="D275" s="2" t="s">
         <v>9</v>
@@ -7839,10 +7839,10 @@
     </row>
     <row r="276">
       <c r="A276" s="2" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C276" s="2" t="s">
         <v>321</v>
@@ -7859,7 +7859,7 @@
     </row>
     <row r="277">
       <c r="A277" s="2" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="B277" s="2" t="s">
         <v>409</v>
@@ -7879,7 +7879,7 @@
     </row>
     <row r="278">
       <c r="A278" s="2" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B278" s="2" t="s">
         <v>481</v>
@@ -7899,7 +7899,7 @@
     </row>
     <row r="279">
       <c r="A279" s="2" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B279" s="2" t="s">
         <v>414</v>
@@ -7919,7 +7919,7 @@
     </row>
     <row r="280">
       <c r="A280" s="2" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B280" s="2" t="s">
         <v>416</v>
@@ -7939,7 +7939,7 @@
     </row>
     <row r="281">
       <c r="A281" s="2" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B281" s="2" t="s">
         <v>421</v>
@@ -7959,7 +7959,7 @@
     </row>
     <row r="282">
       <c r="A282" s="2" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B282" s="2" t="s">
         <v>424</v>
@@ -7979,7 +7979,7 @@
     </row>
     <row r="283">
       <c r="A283" s="2" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="B283" s="2" t="s">
         <v>7</v>
@@ -7999,10 +7999,10 @@
     </row>
     <row r="284">
       <c r="A284" s="2" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="C284" s="2" t="s">
         <v>8</v>
@@ -8019,10 +8019,10 @@
     </row>
     <row r="285">
       <c r="A285" s="2" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="C285" s="2" t="s">
         <v>8</v>
@@ -8039,10 +8039,10 @@
     </row>
     <row r="286">
       <c r="A286" s="2" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="C286" s="2" t="s">
         <v>8</v>
@@ -8059,10 +8059,10 @@
     </row>
     <row r="287">
       <c r="A287" s="2" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="C287" s="2" t="s">
         <v>8</v>
@@ -8079,10 +8079,10 @@
     </row>
     <row r="288">
       <c r="A288" s="2" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="C288" s="2" t="s">
         <v>8</v>
@@ -8099,10 +8099,10 @@
     </row>
     <row r="289">
       <c r="A289" s="2" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="C289" s="2" t="s">
         <v>8</v>
@@ -8119,10 +8119,10 @@
     </row>
     <row r="290">
       <c r="A290" s="2" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C290" s="2" t="s">
         <v>8</v>
@@ -8139,10 +8139,10 @@
     </row>
     <row r="291">
       <c r="A291" s="2" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="C291" s="2" t="s">
         <v>8</v>
@@ -8159,10 +8159,10 @@
     </row>
     <row r="292">
       <c r="A292" s="2" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="C292" s="2" t="s">
         <v>8</v>
@@ -8179,10 +8179,10 @@
     </row>
     <row r="293">
       <c r="A293" s="2" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="B293" s="2" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="C293" s="2" t="s">
         <v>8</v>
@@ -8199,10 +8199,10 @@
     </row>
     <row r="294">
       <c r="A294" s="2" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B294" s="2" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C294" s="2" t="s">
         <v>321</v>
@@ -8219,10 +8219,10 @@
     </row>
     <row r="295">
       <c r="A295" s="2" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B295" s="2" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="C295" s="2" t="s">
         <v>321</v>
@@ -8239,10 +8239,10 @@
     </row>
     <row r="296">
       <c r="A296" s="2" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B296" s="2" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="C296" s="2" t="s">
         <v>8</v>
@@ -8259,10 +8259,10 @@
     </row>
     <row r="297">
       <c r="A297" s="2" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="C297" s="2" t="s">
         <v>8</v>
@@ -8279,10 +8279,10 @@
     </row>
     <row r="298">
       <c r="A298" s="2" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="C298" s="2" t="s">
         <v>8</v>
@@ -8299,10 +8299,10 @@
     </row>
     <row r="299">
       <c r="A299" s="2" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B299" s="2" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="C299" s="2" t="s">
         <v>8</v>
@@ -8319,10 +8319,10 @@
     </row>
     <row r="300">
       <c r="A300" s="2" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B300" s="2" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="C300" s="2" t="s">
         <v>8</v>
@@ -8339,10 +8339,10 @@
     </row>
     <row r="301">
       <c r="A301" s="2" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B301" s="2" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="C301" s="2" t="s">
         <v>8</v>
@@ -8359,10 +8359,10 @@
     </row>
     <row r="302">
       <c r="A302" s="2" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B302" s="2" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="C302" s="2" t="s">
         <v>321</v>
@@ -8379,10 +8379,10 @@
     </row>
     <row r="303">
       <c r="A303" s="2" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B303" s="2" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="C303" s="2" t="s">
         <v>339</v>
@@ -8399,13 +8399,13 @@
     </row>
     <row r="304">
       <c r="A304" s="2" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="B304" s="2" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="C304" s="2" t="s">
-        <v>620</v>
+        <v>520</v>
       </c>
       <c r="D304" s="2" t="s">
         <v>9</v>

</xml_diff>